<commit_message>
Regenera binarios do Kit com as correcoes (narrado + normas + ABNT + conservador)
Regenerados a partir dos geradores ja corrigidos e RE-TESTADOS:
- 4 ferramentas (LITE+PRO) e slides: sem Grupo VIP, calibragem conservadora
  (Defesa Civil 199/Bombeiros 193), edicoes de norma.
- 4 planilhas .xlsx: testadas (formulas lib) — 4/4 suites PASSARAM.
- 4 ferramentas .html: testadas (node vm) — 4/4 suites PASSARAM.
- 24 PDFs do Kit (apostila/checklist/guia-bolso/ebook/laudos) via Chromium headless.
- 4 fluxogramas .svg regenerados do .mmd (mermaid-cli) com edicoes de norma.
- 5 .docx (laudos/termos) regenerados.
- Apostilas com nota de direito autoral ABNT.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018F8nc2s9uRgxM8v4RubvM1
</commit_message>
<xml_diff>
--- a/escola-de-obra/04-curso-fundacoes/kit/planilha/planilha-fundacoes.xlsx
+++ b/escola-de-obra/04-curso-fundacoes/kit/planilha/planilha-fundacoes.xlsx
@@ -783,7 +783,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SELETOR DE FUNDAÇÃO — triagem por caso (decisão final: projetista de fundações, NBR 6122)</t>
+          <t>SELETOR DE FUNDAÇÃO — triagem por caso (decisão final: projetista de fundações, NBR 6122:2019)</t>
         </is>
       </c>
     </row>
@@ -3042,7 +3042,7 @@
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>NBR 6122</t>
+          <t>NBR 6122:2019</t>
         </is>
       </c>
     </row>
@@ -3069,7 +3069,7 @@
       </c>
       <c r="E4" s="13" t="inlineStr">
         <is>
-          <t>NBR 6122</t>
+          <t>NBR 6122:2019</t>
         </is>
       </c>
     </row>
@@ -3096,7 +3096,7 @@
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>NBR 6122</t>
+          <t>NBR 6122:2019</t>
         </is>
       </c>
     </row>
@@ -3123,7 +3123,7 @@
       </c>
       <c r="E6" s="13" t="inlineStr">
         <is>
-          <t>NBR 6122</t>
+          <t>NBR 6122:2019</t>
         </is>
       </c>
     </row>
@@ -3150,7 +3150,7 @@
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>NBR 6122</t>
+          <t>NBR 6122:2019</t>
         </is>
       </c>
     </row>
@@ -3177,7 +3177,7 @@
       </c>
       <c r="E8" s="13" t="inlineStr">
         <is>
-          <t>NBR 6122</t>
+          <t>NBR 6122:2019</t>
         </is>
       </c>
     </row>
@@ -3204,7 +3204,7 @@
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>NBR 6122</t>
+          <t>NBR 6122:2019</t>
         </is>
       </c>
     </row>
@@ -3231,7 +3231,7 @@
       </c>
       <c r="E10" s="13" t="inlineStr">
         <is>
-          <t>NBR 6122</t>
+          <t>NBR 6122:2019</t>
         </is>
       </c>
     </row>
@@ -3258,7 +3258,7 @@
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>NBR 6122</t>
+          <t>NBR 6122:2019</t>
         </is>
       </c>
     </row>
@@ -3285,7 +3285,7 @@
       </c>
       <c r="E12" s="13" t="inlineStr">
         <is>
-          <t>NBR 6122</t>
+          <t>NBR 6122:2019</t>
         </is>
       </c>
     </row>
@@ -3312,7 +3312,7 @@
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>NBR 6122</t>
+          <t>NBR 6122:2019</t>
         </is>
       </c>
     </row>
@@ -3339,7 +3339,7 @@
       </c>
       <c r="E14" s="13" t="inlineStr">
         <is>
-          <t>NBR 6122</t>
+          <t>NBR 6122:2019</t>
         </is>
       </c>
     </row>
@@ -3366,7 +3366,7 @@
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>NBR 6122</t>
+          <t>NBR 6122:2019</t>
         </is>
       </c>
     </row>
@@ -3393,7 +3393,7 @@
       </c>
       <c r="E16" s="13" t="inlineStr">
         <is>
-          <t>NBR 6122 / NR</t>
+          <t>NBR 6122:2019 / NR</t>
         </is>
       </c>
     </row>
@@ -3479,7 +3479,7 @@
     <row r="6">
       <c r="A6" s="23" t="inlineStr">
         <is>
-          <t>Como usar: preencha o Seletor (uma linha por apoio/situação). Família, tipos candidatos e alerta são calculados a partir dos Parametros. TODA escolha é uma triagem — a decisão e o dimensionamento finais são do projetista de fundações (NBR 6122).</t>
+          <t>Como usar: preencha o Seletor (uma linha por apoio/situação). Família, tipos candidatos e alerta são calculados a partir dos Parametros. TODA escolha é uma triagem — a decisão e o dimensionamento finais são do projetista de fundações (NBR 6122:2019).</t>
         </is>
       </c>
     </row>

</xml_diff>